<commit_message>
Update site pages, components, and data
</commit_message>
<xml_diff>
--- a/src/data/blogs.xlsx
+++ b/src/data/blogs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\h2oontherock8\Projects\alexyaphomes\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B3A5E0-DEAD-487A-AA9B-90B26068D767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC19228E-E5B3-4CC6-ACF9-4372D641289C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9640" yWindow="3250" windowWidth="26980" windowHeight="17510" xr2:uid="{EA127BBB-0D1C-4335-92AB-5909B3AEAC9B}"/>
+    <workbookView xWindow="6530" yWindow="3580" windowWidth="26980" windowHeight="17510" xr2:uid="{EA127BBB-0D1C-4335-92AB-5909B3AEAC9B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="34">
   <si>
     <t>title</t>
   </si>
@@ -89,12 +89,6 @@
   </si>
   <si>
     <t>Full paragraph text goes here...</t>
-  </si>
-  <si>
-    <t>North Bay Real Estate Trends for 2026</t>
-  </si>
-  <si>
-    <t>West Bay Real Estate Trends for 2026</t>
   </si>
   <si>
     <t>East Bay Real Estate Trends for 2026</t>
@@ -150,9 +144,6 @@
   </si>
   <si>
     <t>San Jose</t>
-  </si>
-  <si>
-    <t>Cupertino</t>
   </si>
   <si>
     <t>Mountain View</t>
@@ -680,7 +671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB926D22-6483-47A0-A2DC-C8984312C4BF}">
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="13.08984375" style="14" customWidth="1"/>
@@ -688,17 +679,18 @@
     <col min="4" max="4" width="9.7265625" customWidth="1"/>
     <col min="5" max="5" width="14.36328125" customWidth="1"/>
     <col min="6" max="6" width="48.26953125" customWidth="1"/>
-    <col min="7" max="7" width="30.54296875" customWidth="1"/>
-    <col min="8" max="8" width="38" customWidth="1"/>
-    <col min="9" max="9" width="49.36328125" customWidth="1"/>
+    <col min="7" max="7" width="11.26953125" customWidth="1"/>
+    <col min="8" max="8" width="30.54296875" customWidth="1"/>
+    <col min="9" max="9" width="38" customWidth="1"/>
+    <col min="10" max="10" width="49.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>0</v>
@@ -712,119 +704,132 @@
       <c r="F1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="15"/>
+      <c r="H1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="20">
         <f>MAX(A3:A1000) + 1</f>
         <v>7</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D2" s="18">
         <v>46307</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F2" s="16" t="str" cm="1">
-        <f t="array" ref="F2">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.raw, B2 &amp; " " &amp; C2, _xlpm.clean, SUBSTITUTE(SUBSTITUTE(_xlpm.raw, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-")) &amp; "-" &amp; TEXT(D2, "yyyy-mm-dd")</f>
-        <v>san-jose-south-bay-real-estate-trends-for-2026-2026-10-12</v>
-      </c>
-      <c r="G2" s="3" t="s">
+        <f t="array" ref="F2">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.clean, SUBSTITUTE(SUBSTITUTE(C2, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-")) &amp; "-" &amp; TEXT(D2, "yyyy-mm-dd")</f>
+        <v>south-bay-real-estate-trends-for-2026-2026-10-12</v>
+      </c>
+      <c r="G2" s="16" t="str">
+        <f t="shared" ref="G2:G3" si="0">IF(COUNTIF(F:F, F2) &gt; 1, "Yes", "---")</f>
+        <v>Yes</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="I2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="21">
-        <f t="shared" ref="A3:A8" si="0">MAX(A4:A1001) + 1</f>
+        <f t="shared" ref="A3:A8" si="1">MAX(A4:A1001) + 1</f>
         <v>6</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="D3" s="19">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F3" s="17" t="str" cm="1">
         <f t="array" ref="F3">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.clean, SUBSTITUTE(SUBSTITUTE(C3, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-")) &amp; "-" &amp; TEXT(D3, "yyyy-mm-dd")</f>
-        <v>north-bay-real-estate-trends-for-2026-2026-10-11</v>
-      </c>
-      <c r="G3" s="8" t="s">
+        <v>south-bay-real-estate-trends-for-2026-2026-10-12</v>
+      </c>
+      <c r="G3" s="17" t="str">
+        <f t="shared" si="0"/>
+        <v>Yes</v>
+      </c>
+      <c r="H3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="I3" s="10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="I3" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="D4" s="18">
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="16" t="str" cm="1">
         <f t="array" ref="F4">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.clean, SUBSTITUTE(SUBSTITUTE(C4, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-")) &amp; "-" &amp; TEXT(D4, "yyyy-mm-dd")</f>
-        <v>west-bay-real-estate-trends-for-2026-2026-10-10</v>
-      </c>
-      <c r="G4" s="5" t="s">
+        <v>south-bay-real-estate-trends-for-2026-2026-10-12</v>
+      </c>
+      <c r="G4" s="16" t="str">
+        <f>IF(COUNTIF(F:F, F4) &gt; 1, "Yes", "---")</f>
+        <v>Yes</v>
+      </c>
+      <c r="H4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="I4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" s="19">
         <v>46304</v>
@@ -836,26 +841,30 @@
         <f t="array" ref="F5">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.clean, SUBSTITUTE(SUBSTITUTE(C5, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-")) &amp; "-" &amp; TEXT(D5, "yyyy-mm-dd")</f>
         <v>east-bay-real-estate-trends-for-2026-2026-10-09</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="17" t="str">
+        <f t="shared" ref="G5:G8" si="2">IF(COUNTIF(F:F, F5) &gt; 1, "Yes", "---")</f>
+        <v>---</v>
+      </c>
+      <c r="H5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="I5" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J5" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="B6" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>34</v>
       </c>
       <c r="D6" s="18">
         <v>46303</v>
@@ -867,26 +876,30 @@
         <f t="array" ref="F6">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.clean, SUBSTITUTE(SUBSTITUTE(C6, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-")) &amp; "-" &amp; TEXT(D6, "yyyy-mm-dd")</f>
         <v>south-bay-real-estate-trends-for-2026-2026-10-08</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v>---</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="I6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I6" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J6" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D7" s="19">
         <v>46302</v>
@@ -898,23 +911,27 @@
         <f t="array" ref="F7">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.clean, SUBSTITUTE(SUBSTITUTE(C7, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-")) &amp; "-" &amp; TEXT(D7, "yyyy-mm-dd")</f>
         <v>south-bay-real-estate-trends-for-2026-2026-10-07</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="17" t="str">
+        <f t="shared" si="2"/>
+        <v>---</v>
+      </c>
+      <c r="H7" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="I7" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="I7" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J7" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>7</v>
@@ -929,50 +946,54 @@
         <f t="array" ref="F8">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.clean, SUBSTITUTE(SUBSTITUTE(C8, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-")) &amp; "-" &amp; TEXT(D8, "yyyy-mm-dd")</f>
         <v>south-bay-real-estate-trends-for-2026-2026-10-06</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v>---</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="I8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I8" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I9" s="1"/>
+      <c r="J8" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="J9" s="1"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I10" s="1"/>
+      <c r="K9" s="1"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="J10" s="1"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I11" s="1"/>
+      <c r="K10" s="1"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="J11" s="1"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I12" s="1"/>
+      <c r="K11" s="1"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="J12" s="1"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I13" s="1"/>
+      <c r="K12" s="1"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="J13" s="1"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I14" s="1"/>
+      <c r="K13" s="1"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="J14" s="1"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I15" s="1"/>
+      <c r="K14" s="1"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="J15" s="1"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I16" s="1"/>
+      <c r="K15" s="1"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="J16" s="1"/>
-    </row>
-    <row r="17" spans="10:10" x14ac:dyDescent="0.35">
-      <c r="J17" s="1"/>
+      <c r="K16" s="1"/>
+    </row>
+    <row r="17" spans="11:11" x14ac:dyDescent="0.35">
+      <c r="K17" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update site pages, components, and all data
</commit_message>
<xml_diff>
--- a/src/data/blogs.xlsx
+++ b/src/data/blogs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\h2oontherock8\Projects\alexyaphomes\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD2C2F67-D0F3-487B-8C0D-AE23296E381C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9691DA42-6B07-4965-B622-0BDBDFF91B9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9580" yWindow="2900" windowWidth="26980" windowHeight="17510" xr2:uid="{EA127BBB-0D1C-4335-92AB-5909B3AEAC9B}"/>
+    <workbookView xWindow="9920" yWindow="3240" windowWidth="26980" windowHeight="17510" xr2:uid="{EA127BBB-0D1C-4335-92AB-5909B3AEAC9B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -292,7 +292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -354,6 +354,11 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -686,6 +691,7 @@
     <col min="8" max="8" width="30.54296875" customWidth="1"/>
     <col min="9" max="9" width="38" customWidth="1"/>
     <col min="10" max="10" width="49.36328125" customWidth="1"/>
+    <col min="11" max="11" width="2.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -717,6 +723,7 @@
       <c r="J1" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="K1" s="22"/>
     </row>
     <row r="2" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="20">
@@ -752,6 +759,7 @@
       <c r="J2" s="4" t="s">
         <v>12</v>
       </c>
+      <c r="K2" s="22"/>
     </row>
     <row r="3" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="21">
@@ -787,6 +795,7 @@
       <c r="J3" s="10" t="s">
         <v>13</v>
       </c>
+      <c r="K3" s="22"/>
     </row>
     <row r="4" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="20">
@@ -822,6 +831,7 @@
       <c r="J4" s="4" t="s">
         <v>14</v>
       </c>
+      <c r="K4" s="22"/>
     </row>
     <row r="5" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="21">
@@ -857,6 +867,7 @@
       <c r="J5" s="10" t="s">
         <v>12</v>
       </c>
+      <c r="K5" s="22"/>
     </row>
     <row r="6" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="20">
@@ -892,6 +903,7 @@
       <c r="J6" s="4" t="s">
         <v>15</v>
       </c>
+      <c r="K6" s="22"/>
     </row>
     <row r="7" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="21">
@@ -927,6 +939,7 @@
       <c r="J7" s="10" t="s">
         <v>16</v>
       </c>
+      <c r="K7" s="22"/>
     </row>
     <row r="8" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="20">
@@ -962,10 +975,20 @@
       <c r="J8" s="4" t="s">
         <v>17</v>
       </c>
+      <c r="K8" s="22"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
+      <c r="A9" s="22"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="24"/>
+      <c r="K9" s="24"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="J10" s="1"/>

</xml_diff>